<commit_message>
members: move Amr Mohamed and Zeph Van Iterson to Alumni
</commit_message>
<xml_diff>
--- a/updates/members/amr-mohamed/info.xlsx
+++ b/updates/members/amr-mohamed/info.xlsx
@@ -497,7 +497,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Graduate</t>
+          <t>Alumni</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -568,7 +568,6 @@
           <t>Joined</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
@@ -577,7 +576,6 @@
           <t>Left</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" s="3" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>